<commit_message>
feat: add SPJ import category column
</commit_message>
<xml_diff>
--- a/public/templates/template_import_spj.xlsx
+++ b/public/templates/template_import_spj.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
   <si>
     <t>No. SP2D</t>
   </si>
@@ -78,6 +78,12 @@
   </si>
   <si>
     <t>UNIT</t>
+  </si>
+  <si>
+    <t>Jenis *</t>
+  </si>
+  <si>
+    <t>Peralatan &amp; Mesin</t>
   </si>
 </sst>
 </file>
@@ -85,7 +91,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -102,6 +108,15 @@
       <u val="none"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -131,10 +146,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -435,24 +453,25 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="24.708" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="47.131" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="41.133" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="30.564" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="10.569" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="16.425" customWidth="true" style="0"/>
+    <col min="2" max="2" width="22.28" customWidth="true" style="0"/>
+    <col min="3" max="3" width="24.708" customWidth="true" style="0"/>
+    <col min="4" max="4" width="47.131" customWidth="true" style="0"/>
+    <col min="5" max="5" width="25.851" customWidth="true" style="0"/>
+    <col min="6" max="6" width="16.425" customWidth="true" style="0"/>
+    <col min="7" max="7" width="23.423" customWidth="true" style="0"/>
+    <col min="8" max="8" width="41.133" customWidth="true" style="0"/>
+    <col min="9" max="9" width="30.564" customWidth="true" style="0"/>
+    <col min="10" max="10" width="10.569" customWidth="true" style="0"/>
+    <col min="11" max="11" width="17.567" customWidth="true" style="0"/>
+    <col min="12" max="12" width="23.423" customWidth="true" style="0"/>
+    <col min="13" max="13" width="24" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -489,8 +508,11 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -523,6 +545,9 @@
       </c>
       <c r="L2">
         <v>7500000</v>
+      </c>
+      <c r="M2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>